<commit_message>
feat(import): add configurable data quality review checks
Add 4 new NEEDS_REVIEW checks that pause imports for human review:
no timestamp field, no location field, high empty row rate (>20%),
and high row error rate (>10%).

Existing checks (high duplicates, geocoding failures) are now
configurable instead of hardcoded. Thresholds set globally via
timetiles.yml, overridable per scheduled-ingest/scraper with skip
flags and custom thresholds in advancedOptions.reviewChecks.

Also gates ingest-files creation behind enableImportCreation flag.
</commit_message>
<xml_diff>
--- a/apps/web/tests/fixtures/multi-sheet.xlsx
+++ b/apps/web/tests/fixtures/multi-sheet.xlsx
@@ -1,54 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Tech Events" sheetId="1" r:id="rId1"/>
-    <sheet name="Art Exhibitions" sheetId="2" r:id="rId2"/>
-    <sheet name="Sports Events" sheetId="3" r:id="rId3"/>
+    <sheet name="Tech Events" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Art Exhibitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sports Events" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -67,13 +44,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -398,247 +442,374 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>title</v>
-      </c>
-      <c r="B1" t="str">
-        <v>event_date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>venue</v>
-      </c>
-      <c r="D1" t="str">
-        <v>city</v>
-      </c>
-      <c r="E1" t="str">
-        <v>description</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>event_date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>AI Summit 2024</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2024-06-15</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Tech Convention Center</v>
-      </c>
-      <c r="D2" t="str">
-        <v>San Francisco, CA</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Annual conference on artificial intelligence trends</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AI Summit 2024</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2024-06-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Tech Convention Center</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Annual conference on artificial intelligence trends</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>Web Dev Conference</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2024-06-20</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Digital Hub</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Austin, TX</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Latest in web development technologies</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Web Dev Conference</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2024-06-20</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Digital Hub</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Latest in web development technologies</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>Startup Pitch Night</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2024-07-01</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Innovation Lab</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Seattle, WA</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Early-stage startups present to investors</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Startup Pitch Night</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2024-07-01</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Innovation Lab</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Early-stage startups present to investors</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>location</v>
-      </c>
-      <c r="D1" t="str">
-        <v>details</v>
-      </c>
-      <c r="E1" t="str">
-        <v>category</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>details</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Modern Masters Exhibition</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2024-07-10</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Metropolitan Art Museum, New York, NY</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Collection of 20th century masterpieces</v>
-      </c>
-      <c r="E2" t="str">
-        <v>painting</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Modern Masters Exhibition</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2024-07-10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Metropolitan Art Museum, New York, NY</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Collection of 20th century masterpieces</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>painting</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>Sculpture Garden Opening</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2024-07-15</v>
-      </c>
-      <c r="C3" t="str">
-        <v>City Sculpture Park, Chicago, IL</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Outdoor exhibition of contemporary sculptures</v>
-      </c>
-      <c r="E3" t="str">
-        <v>sculpture</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sculpture Garden Opening</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2024-07-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>City Sculpture Park, Chicago, IL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Outdoor exhibition of contemporary sculptures</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>sculpture</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>Photography Retrospective</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2024-08-01</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Gallery of Fine Arts, Los Angeles, CA</v>
-      </c>
-      <c r="D4" t="str">
-        <v>50 years of documentary photography</v>
-      </c>
-      <c r="E4" t="str">
-        <v>photography</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Photography Retrospective</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2024-08-01</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Gallery of Fine Arts, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>50 years of documentary photography</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>photography</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>Digital Art Fair</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2024-08-10</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Creative Center, Miami, FL</v>
-      </c>
-      <c r="D5" t="str">
-        <v>NFTs and digital installations</v>
-      </c>
-      <c r="E5" t="str">
-        <v>digital</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Digital Art Fair</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2024-08-10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Creative Center, Miami, FL</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NFTs and digital installations</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>digital</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>event_name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>start_date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>address</v>
-      </c>
-      <c r="D1" t="str">
-        <v>lat</v>
-      </c>
-      <c r="E1" t="str">
-        <v>lng</v>
-      </c>
-      <c r="F1" t="str">
-        <v>notes</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>event_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>lng</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>City Marathon</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2024-09-01</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Central Park, New York, NY</v>
-      </c>
-      <c r="D2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>City Marathon</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2024-09-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Central Park, New York, NY</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>40.7829</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>-73.9654</v>
       </c>
-      <c r="F2" t="str">
-        <v>Annual 26.2 mile race through the city</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Annual 26.2 mile race through the city</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>Tennis Open</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2024-09-15</v>
-      </c>
-      <c r="C3" t="str">
-        <v>National Tennis Center, Flushing, NY</v>
-      </c>
-      <c r="D3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tennis Open</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2024-09-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>National Tennis Center, Flushing, NY</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>40.7498</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>-73.8477</v>
       </c>
-      <c r="F3" t="str">
-        <v>Professional tennis tournament</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Professional tennis tournament</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>